<commit_message>
Update Philly BYOB Restaurant_with_google_yelp_20251108_153121.xlsx
</commit_message>
<xml_diff>
--- a/philly_yelp_crawler/data/Philly BYOB Restaurant_with_google_yelp_20251108_153121.xlsx
+++ b/philly_yelp_crawler/data/Philly BYOB Restaurant_with_google_yelp_20251108_153121.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\slow3\OneDrive\桌面\GitHubProjects\BYOB\philly_yelp_crawler\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AF9FA35-4054-48A3-9BCF-98B5289EE8F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{318EBEA2-8316-4199-B858-D2589E628FD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -94,9 +94,6 @@
     <t>Ambrosia Ristorante</t>
   </si>
   <si>
-    <t>231 S 24th St, Philadelphia, PA 19103, United States</t>
-  </si>
-  <si>
     <t>(215) 703-2010</t>
   </si>
   <si>
@@ -109,9 +106,6 @@
     <t>Bistro La Baia BYOB</t>
   </si>
   <si>
-    <t>1700 Lombard St, Philadelphia, PA 19146, United States</t>
-  </si>
-  <si>
     <t>(267) 687-1561</t>
   </si>
   <si>
@@ -127,9 +121,6 @@
     <t>Burrata</t>
   </si>
   <si>
-    <t>1247 S 13th St, Philadelphia, PA 19147, United States</t>
-  </si>
-  <si>
     <t>(215) 465-2200</t>
   </si>
   <si>
@@ -199,9 +190,6 @@
     <t>Giorgio On Pine</t>
   </si>
   <si>
-    <t>1328 Pine St, Philadelphia, PA 19107, United States</t>
-  </si>
-  <si>
     <t>(215) 545-6265</t>
   </si>
   <si>
@@ -214,9 +202,6 @@
     <t>Giorgio on Pine II</t>
   </si>
   <si>
-    <t>1334 Pine St, Philadelphia, PA 19107, United States</t>
-  </si>
-  <si>
     <t>(215) 545-2482</t>
   </si>
   <si>
@@ -226,9 +211,6 @@
     <t>Helm</t>
   </si>
   <si>
-    <t>1303 N 5th St, Philadelphia, PA 19122, United States</t>
-  </si>
-  <si>
     <t>(215) 309-2211</t>
   </si>
   <si>
@@ -256,9 +238,6 @@
     <t>ILLATA</t>
   </si>
   <si>
-    <t>2241 Grays Ferry Ave, Philadelphia, PA 19146, United States</t>
-  </si>
-  <si>
     <t>2241 Grays Ferry Ave, Philadelphia, PA 19146美國</t>
   </si>
   <si>
@@ -268,9 +247,6 @@
     <t>Kei Sushi</t>
   </si>
   <si>
-    <t>1711 South St, Philadelphia, PA 19146, United States</t>
-  </si>
-  <si>
     <t>(215) 309-2925</t>
   </si>
   <si>
@@ -286,9 +262,6 @@
     <t>Kichi Omakase</t>
   </si>
   <si>
-    <t>112 S 12th St, Philadelphia, PA 19107, United States</t>
-  </si>
-  <si>
     <t>(215) 359-6099</t>
   </si>
   <si>
@@ -301,9 +274,6 @@
     <t>Kinme</t>
   </si>
   <si>
-    <t>1117 Locust St, Philadelphia, PA 19107, United States</t>
-  </si>
-  <si>
     <t>(215) 982-1722</t>
   </si>
   <si>
@@ -349,9 +319,6 @@
     <t>La Sera Italiana BYOB</t>
   </si>
   <si>
-    <t>1608 South St, Philadelphia, PA 19146, United States</t>
-  </si>
-  <si>
     <t>(267) 930-7805</t>
   </si>
   <si>
@@ -361,9 +328,6 @@
     <t>La Viola Bistro</t>
   </si>
   <si>
-    <t>253 S 16th St, Philadelphia, PA 19102, United States</t>
-  </si>
-  <si>
     <t>(215) 735-8630</t>
   </si>
   <si>
@@ -376,9 +340,6 @@
     <t>L'Angolo Ristorante</t>
   </si>
   <si>
-    <t>1415 W Porter St, Philadelphia, PA 19145, United States</t>
-  </si>
-  <si>
     <t>(215) 389-4252</t>
   </si>
   <si>
@@ -391,9 +352,6 @@
     <t>L'Anima</t>
   </si>
   <si>
-    <t>1001 S 17th St, Philadelphia, PA 19146, United States</t>
-  </si>
-  <si>
     <t>(215) 595-2500</t>
   </si>
   <si>
@@ -421,9 +379,6 @@
     <t>Luna BYOB</t>
   </si>
   <si>
-    <t>227 S 20th St, Philadelphia, PA 19103, United States</t>
-  </si>
-  <si>
     <t>(215) 693-2220</t>
   </si>
   <si>
@@ -448,9 +403,6 @@
     <t>Melograno</t>
   </si>
   <si>
-    <t>2012 Sansom St, Philadelphia, PA 19103, United States</t>
-  </si>
-  <si>
     <t>(215) 875-8116</t>
   </si>
   <si>
@@ -463,9 +415,6 @@
     <t>Mercato</t>
   </si>
   <si>
-    <t>1216 Spruce St, Philadelphia, PA 19107, United States</t>
-  </si>
-  <si>
     <t>(215) 985-2962</t>
   </si>
   <si>
@@ -493,9 +442,6 @@
     <t>Nori Sushi</t>
   </si>
   <si>
-    <t>1636 South St, Philadelphia, PA 19146, United States</t>
-  </si>
-  <si>
     <t>(215) 735-6668</t>
   </si>
   <si>
@@ -586,9 +532,6 @@
     <t>Sawatdee</t>
   </si>
   <si>
-    <t>534 S 15th St, Philadelphia, PA 19146, United States</t>
-  </si>
-  <si>
     <t>(215) 790-1299</t>
   </si>
   <si>
@@ -646,9 +589,6 @@
     <t>Thai Square Restaurant</t>
   </si>
   <si>
-    <t>2521 Christian St, Philadelphia, PA 19146, United States</t>
-  </si>
-  <si>
     <t>(215) 454-6683</t>
   </si>
   <si>
@@ -661,9 +601,6 @@
     <t>Trattoria Carina</t>
   </si>
   <si>
-    <t>2201 Spruce St, Philadelphia, PA 19103, United States</t>
-  </si>
-  <si>
     <t>(215) 732-5818</t>
   </si>
   <si>
@@ -704,6 +641,69 @@
   </si>
   <si>
     <t>https://www.yelp.com/biz/vientiane-caf%C3%A9-philadelphia-3</t>
+  </si>
+  <si>
+    <t>1700 Lombard St, Philadelphia, PA 19146</t>
+  </si>
+  <si>
+    <t>1247 S 13th St, Philadelphia, PA 19147</t>
+  </si>
+  <si>
+    <t>1328 Pine St, Philadelphia, PA 19107</t>
+  </si>
+  <si>
+    <t>1334 Pine St, Philadelphia, PA 19107</t>
+  </si>
+  <si>
+    <t>1303 N 5th St, Philadelphia, PA 19122</t>
+  </si>
+  <si>
+    <t>2241 Grays Ferry Ave, Philadelphia, PA 19146</t>
+  </si>
+  <si>
+    <t>1711 South St, Philadelphia, PA 19146</t>
+  </si>
+  <si>
+    <t>112 S 12th St, Philadelphia, PA 19107</t>
+  </si>
+  <si>
+    <t>1117 Locust St, Philadelphia, PA 19107</t>
+  </si>
+  <si>
+    <t>1608 South St, Philadelphia, PA 19146</t>
+  </si>
+  <si>
+    <t>253 S 16th St, Philadelphia, PA 19102</t>
+  </si>
+  <si>
+    <t>1415 W Porter St, Philadelphia, PA 19145</t>
+  </si>
+  <si>
+    <t>1001 S 17th St, Philadelphia, PA 19146</t>
+  </si>
+  <si>
+    <t>227 S 20th St, Philadelphia, PA 19103</t>
+  </si>
+  <si>
+    <t>2012 Sansom St, Philadelphia, PA 19103</t>
+  </si>
+  <si>
+    <t>1216 Spruce St, Philadelphia, PA 19107</t>
+  </si>
+  <si>
+    <t>1636 South St, Philadelphia, PA 19146</t>
+  </si>
+  <si>
+    <t>534 S 15th St, Philadelphia, PA 19146</t>
+  </si>
+  <si>
+    <t>2521 Christian St, Philadelphia, PA 19146</t>
+  </si>
+  <si>
+    <t>2201 Spruce St, Philadelphia, PA 19103</t>
+  </si>
+  <si>
+    <t>231 S 24th St, Philadelphia, PA 19103</t>
   </si>
 </sst>
 </file>
@@ -1079,6 +1079,7 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="19.125" customWidth="1"/>
+    <col min="3" max="3" width="20.5" customWidth="1"/>
     <col min="5" max="5" width="27.75" customWidth="1"/>
     <col min="8" max="8" width="22.25" customWidth="1"/>
   </cols>
@@ -1178,22 +1179,22 @@
         <v>23</v>
       </c>
       <c r="B4" t="s">
+        <v>227</v>
+      </c>
+      <c r="C4" t="s">
         <v>24</v>
-      </c>
-      <c r="C4" t="s">
-        <v>25</v>
       </c>
       <c r="D4" t="s">
         <v>23</v>
       </c>
       <c r="E4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F4" t="s">
+        <v>14</v>
+      </c>
+      <c r="H4" t="s">
         <v>26</v>
-      </c>
-      <c r="F4" t="s">
-        <v>14</v>
-      </c>
-      <c r="H4" t="s">
-        <v>27</v>
       </c>
       <c r="I4" t="s">
         <v>16</v>
@@ -1204,51 +1205,51 @@
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
+        <v>27</v>
+      </c>
+      <c r="B5" t="s">
+        <v>207</v>
+      </c>
+      <c r="C5" t="s">
         <v>28</v>
       </c>
-      <c r="B5" t="s">
+      <c r="D5" t="s">
+        <v>27</v>
+      </c>
+      <c r="E5" t="s">
         <v>29</v>
       </c>
-      <c r="C5" t="s">
+      <c r="F5" t="s">
+        <v>14</v>
+      </c>
+      <c r="I5" t="s">
         <v>30</v>
       </c>
-      <c r="D5" t="s">
-        <v>28</v>
-      </c>
-      <c r="E5" t="s">
+      <c r="J5" t="s">
         <v>31</v>
-      </c>
-      <c r="F5" t="s">
-        <v>14</v>
-      </c>
-      <c r="I5" t="s">
-        <v>32</v>
-      </c>
-      <c r="J5" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
+        <v>32</v>
+      </c>
+      <c r="B6" t="s">
+        <v>208</v>
+      </c>
+      <c r="C6" t="s">
+        <v>33</v>
+      </c>
+      <c r="D6" t="s">
+        <v>32</v>
+      </c>
+      <c r="E6" t="s">
         <v>34</v>
       </c>
-      <c r="B6" t="s">
+      <c r="F6" t="s">
+        <v>14</v>
+      </c>
+      <c r="H6" t="s">
         <v>35</v>
-      </c>
-      <c r="C6" t="s">
-        <v>36</v>
-      </c>
-      <c r="D6" t="s">
-        <v>34</v>
-      </c>
-      <c r="E6" t="s">
-        <v>37</v>
-      </c>
-      <c r="F6" t="s">
-        <v>14</v>
-      </c>
-      <c r="H6" t="s">
-        <v>38</v>
       </c>
       <c r="I6" t="s">
         <v>16</v>
@@ -1259,25 +1260,25 @@
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
+        <v>36</v>
+      </c>
+      <c r="B7" t="s">
+        <v>37</v>
+      </c>
+      <c r="C7" t="s">
+        <v>38</v>
+      </c>
+      <c r="D7" t="s">
+        <v>36</v>
+      </c>
+      <c r="E7" t="s">
         <v>39</v>
       </c>
-      <c r="B7" t="s">
+      <c r="F7" t="s">
+        <v>14</v>
+      </c>
+      <c r="H7" t="s">
         <v>40</v>
-      </c>
-      <c r="C7" t="s">
-        <v>41</v>
-      </c>
-      <c r="D7" t="s">
-        <v>39</v>
-      </c>
-      <c r="E7" t="s">
-        <v>42</v>
-      </c>
-      <c r="F7" t="s">
-        <v>14</v>
-      </c>
-      <c r="H7" t="s">
-        <v>43</v>
       </c>
       <c r="I7" t="s">
         <v>16</v>
@@ -1288,25 +1289,25 @@
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
+        <v>41</v>
+      </c>
+      <c r="B8" t="s">
+        <v>42</v>
+      </c>
+      <c r="C8" t="s">
+        <v>43</v>
+      </c>
+      <c r="D8" t="s">
+        <v>41</v>
+      </c>
+      <c r="E8" t="s">
         <v>44</v>
       </c>
-      <c r="B8" t="s">
+      <c r="F8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H8" t="s">
         <v>45</v>
-      </c>
-      <c r="C8" t="s">
-        <v>46</v>
-      </c>
-      <c r="D8" t="s">
-        <v>44</v>
-      </c>
-      <c r="E8" t="s">
-        <v>47</v>
-      </c>
-      <c r="F8" t="s">
-        <v>14</v>
-      </c>
-      <c r="H8" t="s">
-        <v>48</v>
       </c>
       <c r="I8" t="s">
         <v>16</v>
@@ -1317,51 +1318,51 @@
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
+        <v>46</v>
+      </c>
+      <c r="B9" t="s">
+        <v>47</v>
+      </c>
+      <c r="C9" t="s">
+        <v>48</v>
+      </c>
+      <c r="D9" t="s">
+        <v>46</v>
+      </c>
+      <c r="E9" t="s">
         <v>49</v>
       </c>
-      <c r="B9" t="s">
-        <v>50</v>
-      </c>
-      <c r="C9" t="s">
-        <v>51</v>
-      </c>
-      <c r="D9" t="s">
-        <v>49</v>
-      </c>
-      <c r="E9" t="s">
-        <v>52</v>
-      </c>
       <c r="F9" t="s">
         <v>14</v>
       </c>
       <c r="I9" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="J9" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
+        <v>50</v>
+      </c>
+      <c r="B10" t="s">
+        <v>51</v>
+      </c>
+      <c r="C10" t="s">
+        <v>52</v>
+      </c>
+      <c r="D10" t="s">
+        <v>50</v>
+      </c>
+      <c r="E10" t="s">
         <v>53</v>
       </c>
-      <c r="B10" t="s">
+      <c r="F10" t="s">
+        <v>14</v>
+      </c>
+      <c r="H10" t="s">
         <v>54</v>
-      </c>
-      <c r="C10" t="s">
-        <v>55</v>
-      </c>
-      <c r="D10" t="s">
-        <v>53</v>
-      </c>
-      <c r="E10" t="s">
-        <v>56</v>
-      </c>
-      <c r="F10" t="s">
-        <v>14</v>
-      </c>
-      <c r="H10" t="s">
-        <v>57</v>
       </c>
       <c r="I10" t="s">
         <v>16</v>
@@ -1372,25 +1373,25 @@
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
+        <v>55</v>
+      </c>
+      <c r="B11" t="s">
+        <v>209</v>
+      </c>
+      <c r="C11" t="s">
+        <v>56</v>
+      </c>
+      <c r="D11" t="s">
+        <v>55</v>
+      </c>
+      <c r="E11" t="s">
+        <v>57</v>
+      </c>
+      <c r="F11" t="s">
+        <v>14</v>
+      </c>
+      <c r="H11" t="s">
         <v>58</v>
-      </c>
-      <c r="B11" t="s">
-        <v>59</v>
-      </c>
-      <c r="C11" t="s">
-        <v>60</v>
-      </c>
-      <c r="D11" t="s">
-        <v>58</v>
-      </c>
-      <c r="E11" t="s">
-        <v>61</v>
-      </c>
-      <c r="F11" t="s">
-        <v>14</v>
-      </c>
-      <c r="H11" t="s">
-        <v>62</v>
       </c>
       <c r="I11" t="s">
         <v>16</v>
@@ -1401,25 +1402,25 @@
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="B12" t="s">
-        <v>64</v>
+        <v>210</v>
       </c>
       <c r="C12" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="D12" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="E12" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="F12" t="s">
         <v>14</v>
       </c>
       <c r="H12" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="I12" t="s">
         <v>16</v>
@@ -1430,25 +1431,25 @@
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="B13" t="s">
-        <v>68</v>
+        <v>211</v>
       </c>
       <c r="C13" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="D13" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="E13" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="F13" t="s">
         <v>14</v>
       </c>
       <c r="H13" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="I13" t="s">
         <v>16</v>
@@ -1459,25 +1460,25 @@
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="B14" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="C14" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="D14" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="E14" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="F14" t="s">
         <v>14</v>
       </c>
       <c r="H14" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="I14" t="s">
         <v>16</v>
@@ -1488,25 +1489,25 @@
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="B15" t="s">
-        <v>78</v>
+        <v>212</v>
       </c>
       <c r="C15" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="D15" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="E15" t="s">
-        <v>79</v>
+        <v>72</v>
       </c>
       <c r="F15" t="s">
         <v>14</v>
       </c>
       <c r="H15" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="I15" t="s">
         <v>16</v>
@@ -1517,25 +1518,25 @@
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>81</v>
+        <v>74</v>
       </c>
       <c r="B16" t="s">
-        <v>82</v>
+        <v>213</v>
       </c>
       <c r="C16" t="s">
-        <v>83</v>
+        <v>75</v>
       </c>
       <c r="D16" t="s">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="E16" t="s">
-        <v>85</v>
+        <v>77</v>
       </c>
       <c r="F16" t="s">
         <v>14</v>
       </c>
       <c r="H16" t="s">
-        <v>86</v>
+        <v>78</v>
       </c>
       <c r="I16" t="s">
         <v>16</v>
@@ -1546,25 +1547,25 @@
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>87</v>
+        <v>79</v>
       </c>
       <c r="B17" t="s">
-        <v>88</v>
+        <v>214</v>
       </c>
       <c r="C17" t="s">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="D17" t="s">
-        <v>87</v>
+        <v>79</v>
       </c>
       <c r="E17" t="s">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="F17" t="s">
         <v>14</v>
       </c>
       <c r="H17" t="s">
-        <v>91</v>
+        <v>82</v>
       </c>
       <c r="I17" t="s">
         <v>16</v>
@@ -1575,25 +1576,25 @@
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>92</v>
+        <v>83</v>
       </c>
       <c r="B18" t="s">
-        <v>93</v>
+        <v>215</v>
       </c>
       <c r="C18" t="s">
-        <v>94</v>
+        <v>84</v>
       </c>
       <c r="D18" t="s">
-        <v>92</v>
+        <v>83</v>
       </c>
       <c r="E18" t="s">
-        <v>95</v>
+        <v>85</v>
       </c>
       <c r="F18" t="s">
         <v>14</v>
       </c>
       <c r="H18" t="s">
-        <v>96</v>
+        <v>86</v>
       </c>
       <c r="I18" t="s">
         <v>16</v>
@@ -1604,54 +1605,54 @@
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="B19" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="C19" t="s">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="D19" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="E19" t="s">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="F19" t="s">
         <v>14</v>
       </c>
       <c r="G19" t="s">
-        <v>101</v>
+        <v>91</v>
       </c>
       <c r="I19" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="J19" t="s">
-        <v>102</v>
+        <v>92</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>103</v>
+        <v>93</v>
       </c>
       <c r="B20" t="s">
-        <v>104</v>
+        <v>94</v>
       </c>
       <c r="C20" t="s">
-        <v>105</v>
+        <v>95</v>
       </c>
       <c r="D20" t="s">
-        <v>103</v>
+        <v>93</v>
       </c>
       <c r="E20" t="s">
-        <v>106</v>
+        <v>96</v>
       </c>
       <c r="F20" t="s">
         <v>14</v>
       </c>
       <c r="H20" t="s">
-        <v>107</v>
+        <v>97</v>
       </c>
       <c r="I20" t="s">
         <v>16</v>
@@ -1662,51 +1663,51 @@
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>108</v>
+        <v>98</v>
       </c>
       <c r="B21" t="s">
-        <v>109</v>
+        <v>216</v>
       </c>
       <c r="C21" t="s">
-        <v>110</v>
+        <v>99</v>
       </c>
       <c r="D21" t="s">
-        <v>108</v>
+        <v>98</v>
       </c>
       <c r="E21" t="s">
-        <v>111</v>
+        <v>100</v>
       </c>
       <c r="F21" t="s">
         <v>14</v>
       </c>
       <c r="I21" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="J21" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>112</v>
+        <v>101</v>
       </c>
       <c r="B22" t="s">
-        <v>113</v>
+        <v>217</v>
       </c>
       <c r="C22" t="s">
-        <v>114</v>
+        <v>102</v>
       </c>
       <c r="D22" t="s">
-        <v>112</v>
+        <v>101</v>
       </c>
       <c r="E22" t="s">
-        <v>115</v>
+        <v>103</v>
       </c>
       <c r="F22" t="s">
         <v>14</v>
       </c>
       <c r="H22" t="s">
-        <v>116</v>
+        <v>104</v>
       </c>
       <c r="I22" t="s">
         <v>16</v>
@@ -1717,25 +1718,25 @@
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>117</v>
+        <v>105</v>
       </c>
       <c r="B23" t="s">
-        <v>118</v>
+        <v>218</v>
       </c>
       <c r="C23" t="s">
-        <v>119</v>
+        <v>106</v>
       </c>
       <c r="D23" t="s">
-        <v>117</v>
+        <v>105</v>
       </c>
       <c r="E23" t="s">
-        <v>120</v>
+        <v>107</v>
       </c>
       <c r="F23" t="s">
         <v>14</v>
       </c>
       <c r="H23" t="s">
-        <v>121</v>
+        <v>108</v>
       </c>
       <c r="I23" t="s">
         <v>16</v>
@@ -1746,28 +1747,28 @@
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>122</v>
+        <v>109</v>
       </c>
       <c r="B24" t="s">
-        <v>123</v>
+        <v>219</v>
       </c>
       <c r="C24" t="s">
-        <v>124</v>
+        <v>110</v>
       </c>
       <c r="D24" t="s">
-        <v>122</v>
+        <v>109</v>
       </c>
       <c r="E24" t="s">
-        <v>125</v>
+        <v>111</v>
       </c>
       <c r="F24" t="s">
         <v>14</v>
       </c>
       <c r="G24" t="s">
-        <v>126</v>
+        <v>112</v>
       </c>
       <c r="H24" t="s">
-        <v>127</v>
+        <v>113</v>
       </c>
       <c r="I24" t="s">
         <v>16</v>
@@ -1778,51 +1779,51 @@
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>128</v>
+        <v>114</v>
       </c>
       <c r="B25" t="s">
-        <v>129</v>
+        <v>115</v>
       </c>
       <c r="C25" t="s">
-        <v>130</v>
+        <v>116</v>
       </c>
       <c r="D25" t="s">
-        <v>128</v>
+        <v>114</v>
       </c>
       <c r="E25" t="s">
-        <v>131</v>
+        <v>117</v>
       </c>
       <c r="F25" t="s">
         <v>14</v>
       </c>
       <c r="I25" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="J25" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>132</v>
+        <v>118</v>
       </c>
       <c r="B26" t="s">
-        <v>133</v>
+        <v>220</v>
       </c>
       <c r="C26" t="s">
-        <v>134</v>
+        <v>119</v>
       </c>
       <c r="D26" t="s">
-        <v>132</v>
+        <v>118</v>
       </c>
       <c r="E26" t="s">
-        <v>135</v>
+        <v>120</v>
       </c>
       <c r="F26" t="s">
         <v>14</v>
       </c>
       <c r="H26" t="s">
-        <v>136</v>
+        <v>121</v>
       </c>
       <c r="I26" t="s">
         <v>16</v>
@@ -1833,25 +1834,25 @@
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>137</v>
+        <v>122</v>
       </c>
       <c r="B27" t="s">
-        <v>138</v>
+        <v>123</v>
       </c>
       <c r="C27" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="D27" t="s">
-        <v>137</v>
+        <v>122</v>
       </c>
       <c r="E27" t="s">
-        <v>139</v>
+        <v>124</v>
       </c>
       <c r="F27" t="s">
         <v>14</v>
       </c>
       <c r="H27" t="s">
-        <v>140</v>
+        <v>125</v>
       </c>
       <c r="I27" t="s">
         <v>16</v>
@@ -1862,28 +1863,28 @@
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>141</v>
+        <v>126</v>
       </c>
       <c r="B28" t="s">
-        <v>142</v>
+        <v>221</v>
       </c>
       <c r="C28" t="s">
-        <v>143</v>
+        <v>127</v>
       </c>
       <c r="D28" t="s">
-        <v>141</v>
+        <v>126</v>
       </c>
       <c r="E28" t="s">
-        <v>144</v>
+        <v>128</v>
       </c>
       <c r="F28" t="s">
         <v>14</v>
       </c>
       <c r="G28" t="s">
-        <v>126</v>
+        <v>112</v>
       </c>
       <c r="H28" t="s">
-        <v>145</v>
+        <v>129</v>
       </c>
       <c r="I28" t="s">
         <v>16</v>
@@ -1894,25 +1895,25 @@
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>146</v>
+        <v>130</v>
       </c>
       <c r="B29" t="s">
-        <v>147</v>
+        <v>222</v>
       </c>
       <c r="C29" t="s">
-        <v>148</v>
+        <v>131</v>
       </c>
       <c r="D29" t="s">
-        <v>146</v>
+        <v>130</v>
       </c>
       <c r="E29" t="s">
-        <v>149</v>
+        <v>132</v>
       </c>
       <c r="F29" t="s">
         <v>14</v>
       </c>
       <c r="H29" t="s">
-        <v>150</v>
+        <v>133</v>
       </c>
       <c r="I29" t="s">
         <v>16</v>
@@ -1923,25 +1924,25 @@
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>151</v>
+        <v>134</v>
       </c>
       <c r="B30" t="s">
-        <v>152</v>
+        <v>135</v>
       </c>
       <c r="C30" t="s">
-        <v>153</v>
+        <v>136</v>
       </c>
       <c r="D30" t="s">
-        <v>151</v>
+        <v>134</v>
       </c>
       <c r="E30" t="s">
-        <v>154</v>
+        <v>137</v>
       </c>
       <c r="F30" t="s">
         <v>14</v>
       </c>
       <c r="H30" t="s">
-        <v>155</v>
+        <v>138</v>
       </c>
       <c r="I30" t="s">
         <v>16</v>
@@ -1952,28 +1953,28 @@
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>156</v>
+        <v>139</v>
       </c>
       <c r="B31" t="s">
-        <v>157</v>
+        <v>223</v>
       </c>
       <c r="C31" t="s">
-        <v>158</v>
+        <v>140</v>
       </c>
       <c r="D31" t="s">
-        <v>156</v>
+        <v>139</v>
       </c>
       <c r="E31" t="s">
-        <v>159</v>
+        <v>141</v>
       </c>
       <c r="F31" t="s">
-        <v>160</v>
+        <v>142</v>
       </c>
       <c r="G31" t="s">
         <v>14</v>
       </c>
       <c r="H31" t="s">
-        <v>161</v>
+        <v>143</v>
       </c>
       <c r="I31" t="s">
         <v>16</v>
@@ -1984,25 +1985,25 @@
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>162</v>
+        <v>144</v>
       </c>
       <c r="B32" t="s">
-        <v>163</v>
+        <v>145</v>
       </c>
       <c r="C32" t="s">
-        <v>164</v>
+        <v>146</v>
       </c>
       <c r="D32" t="s">
-        <v>162</v>
+        <v>144</v>
       </c>
       <c r="E32" t="s">
-        <v>165</v>
+        <v>147</v>
       </c>
       <c r="F32" t="s">
         <v>14</v>
       </c>
       <c r="H32" t="s">
-        <v>166</v>
+        <v>148</v>
       </c>
       <c r="I32" t="s">
         <v>16</v>
@@ -2013,25 +2014,25 @@
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>167</v>
+        <v>149</v>
       </c>
       <c r="B33" t="s">
-        <v>168</v>
+        <v>150</v>
       </c>
       <c r="C33" t="s">
-        <v>169</v>
+        <v>151</v>
       </c>
       <c r="D33" t="s">
-        <v>167</v>
+        <v>149</v>
       </c>
       <c r="E33" t="s">
-        <v>170</v>
+        <v>152</v>
       </c>
       <c r="F33" t="s">
         <v>14</v>
       </c>
       <c r="H33" t="s">
-        <v>171</v>
+        <v>153</v>
       </c>
       <c r="I33" t="s">
         <v>16</v>
@@ -2042,25 +2043,25 @@
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>172</v>
+        <v>154</v>
       </c>
       <c r="B34" t="s">
-        <v>173</v>
+        <v>155</v>
       </c>
       <c r="C34" t="s">
-        <v>174</v>
+        <v>156</v>
       </c>
       <c r="D34" t="s">
-        <v>172</v>
+        <v>154</v>
       </c>
       <c r="E34" t="s">
-        <v>175</v>
+        <v>157</v>
       </c>
       <c r="F34" t="s">
         <v>14</v>
       </c>
       <c r="H34" t="s">
-        <v>176</v>
+        <v>158</v>
       </c>
       <c r="I34" t="s">
         <v>16</v>
@@ -2071,25 +2072,25 @@
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>177</v>
+        <v>159</v>
       </c>
       <c r="B35" t="s">
-        <v>178</v>
+        <v>160</v>
       </c>
       <c r="C35" t="s">
-        <v>179</v>
+        <v>161</v>
       </c>
       <c r="D35" t="s">
-        <v>177</v>
+        <v>159</v>
       </c>
       <c r="E35" t="s">
-        <v>180</v>
+        <v>162</v>
       </c>
       <c r="F35" t="s">
         <v>14</v>
       </c>
       <c r="H35" t="s">
-        <v>181</v>
+        <v>163</v>
       </c>
       <c r="I35" t="s">
         <v>16</v>
@@ -2100,25 +2101,25 @@
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>182</v>
+        <v>164</v>
       </c>
       <c r="B36" t="s">
-        <v>183</v>
+        <v>165</v>
       </c>
       <c r="C36" t="s">
-        <v>184</v>
+        <v>166</v>
       </c>
       <c r="D36" t="s">
-        <v>182</v>
+        <v>164</v>
       </c>
       <c r="E36" t="s">
-        <v>185</v>
+        <v>167</v>
       </c>
       <c r="F36" t="s">
         <v>14</v>
       </c>
       <c r="H36" t="s">
-        <v>186</v>
+        <v>168</v>
       </c>
       <c r="I36" t="s">
         <v>16</v>
@@ -2129,25 +2130,25 @@
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>187</v>
+        <v>169</v>
       </c>
       <c r="B37" t="s">
-        <v>188</v>
+        <v>224</v>
       </c>
       <c r="C37" t="s">
-        <v>189</v>
+        <v>170</v>
       </c>
       <c r="D37" t="s">
-        <v>187</v>
+        <v>169</v>
       </c>
       <c r="E37" t="s">
-        <v>190</v>
+        <v>171</v>
       </c>
       <c r="F37" t="s">
         <v>14</v>
       </c>
       <c r="H37" t="s">
-        <v>191</v>
+        <v>172</v>
       </c>
       <c r="I37" t="s">
         <v>16</v>
@@ -2158,25 +2159,25 @@
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>192</v>
+        <v>173</v>
       </c>
       <c r="B38" t="s">
-        <v>193</v>
+        <v>174</v>
       </c>
       <c r="C38" t="s">
-        <v>194</v>
+        <v>175</v>
       </c>
       <c r="D38" t="s">
-        <v>192</v>
+        <v>173</v>
       </c>
       <c r="E38" t="s">
-        <v>195</v>
+        <v>176</v>
       </c>
       <c r="F38" t="s">
         <v>14</v>
       </c>
       <c r="H38" t="s">
-        <v>196</v>
+        <v>177</v>
       </c>
       <c r="I38" t="s">
         <v>16</v>
@@ -2187,25 +2188,25 @@
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>197</v>
+        <v>178</v>
       </c>
       <c r="B39" t="s">
-        <v>198</v>
+        <v>179</v>
       </c>
       <c r="C39" t="s">
-        <v>199</v>
+        <v>180</v>
       </c>
       <c r="D39" t="s">
-        <v>197</v>
+        <v>178</v>
       </c>
       <c r="E39" t="s">
-        <v>200</v>
+        <v>181</v>
       </c>
       <c r="F39" t="s">
         <v>14</v>
       </c>
       <c r="H39" t="s">
-        <v>201</v>
+        <v>182</v>
       </c>
       <c r="I39" t="s">
         <v>16</v>
@@ -2216,28 +2217,28 @@
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>202</v>
+        <v>183</v>
       </c>
       <c r="B40" t="s">
-        <v>203</v>
+        <v>184</v>
       </c>
       <c r="C40" t="s">
-        <v>204</v>
+        <v>185</v>
       </c>
       <c r="D40" t="s">
-        <v>202</v>
+        <v>183</v>
       </c>
       <c r="E40" t="s">
-        <v>205</v>
+        <v>186</v>
       </c>
       <c r="F40" t="s">
-        <v>160</v>
+        <v>142</v>
       </c>
       <c r="G40" t="s">
         <v>14</v>
       </c>
       <c r="H40" t="s">
-        <v>206</v>
+        <v>187</v>
       </c>
       <c r="I40" t="s">
         <v>16</v>
@@ -2248,25 +2249,25 @@
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>207</v>
+        <v>188</v>
       </c>
       <c r="B41" t="s">
-        <v>208</v>
+        <v>225</v>
       </c>
       <c r="C41" t="s">
-        <v>209</v>
+        <v>189</v>
       </c>
       <c r="D41" t="s">
-        <v>207</v>
+        <v>188</v>
       </c>
       <c r="E41" t="s">
-        <v>210</v>
+        <v>190</v>
       </c>
       <c r="F41" t="s">
         <v>14</v>
       </c>
       <c r="H41" t="s">
-        <v>211</v>
+        <v>191</v>
       </c>
       <c r="I41" t="s">
         <v>16</v>
@@ -2277,25 +2278,25 @@
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>212</v>
+        <v>192</v>
       </c>
       <c r="B42" t="s">
-        <v>213</v>
+        <v>226</v>
       </c>
       <c r="C42" t="s">
-        <v>214</v>
+        <v>193</v>
       </c>
       <c r="D42" t="s">
-        <v>212</v>
+        <v>192</v>
       </c>
       <c r="E42" t="s">
-        <v>215</v>
+        <v>194</v>
       </c>
       <c r="F42" t="s">
         <v>14</v>
       </c>
       <c r="H42" t="s">
-        <v>216</v>
+        <v>195</v>
       </c>
       <c r="I42" t="s">
         <v>16</v>
@@ -2306,25 +2307,25 @@
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>217</v>
+        <v>196</v>
       </c>
       <c r="B43" t="s">
-        <v>218</v>
+        <v>197</v>
       </c>
       <c r="C43" t="s">
-        <v>219</v>
+        <v>198</v>
       </c>
       <c r="D43" t="s">
-        <v>217</v>
+        <v>196</v>
       </c>
       <c r="E43" t="s">
-        <v>220</v>
+        <v>199</v>
       </c>
       <c r="F43" t="s">
         <v>14</v>
       </c>
       <c r="H43" t="s">
-        <v>221</v>
+        <v>200</v>
       </c>
       <c r="I43" t="s">
         <v>16</v>
@@ -2335,28 +2336,28 @@
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>222</v>
+        <v>201</v>
       </c>
       <c r="B44" t="s">
-        <v>223</v>
+        <v>202</v>
       </c>
       <c r="C44" t="s">
-        <v>224</v>
+        <v>203</v>
       </c>
       <c r="D44" t="s">
-        <v>222</v>
+        <v>201</v>
       </c>
       <c r="E44" t="s">
-        <v>225</v>
+        <v>204</v>
       </c>
       <c r="F44" t="s">
-        <v>226</v>
+        <v>205</v>
       </c>
       <c r="G44" t="s">
         <v>14</v>
       </c>
       <c r="H44" t="s">
-        <v>227</v>
+        <v>206</v>
       </c>
       <c r="I44" t="s">
         <v>16</v>

</xml_diff>